<commit_message>
Calculated price-change R^2 for levels models and adapted run_all_models
</commit_message>
<xml_diff>
--- a/Quarter/Lasso_Price_Predictions.xlsx
+++ b/Quarter/Lasso_Price_Predictions.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Model_Summary" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Feature_Importance" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Feature_Description" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Price_Change_R2" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20139,7 +20140,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20655,6 +20656,28 @@
         <v>9</v>
       </c>
       <c r="F23" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Overall (Average)</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1750</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.574524560051934</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.02740565706133723</v>
+      </c>
+      <c r="E24" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="F24" t="n">
         <v>9</v>
       </c>
     </row>
@@ -24395,4 +24418,463 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Interval</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>R2_Price_Change</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Samples</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Mean_Actual_Delta</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Mean_Predicted_Delta</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2020 Q1 → 2020 Q2</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.7240122179279672</v>
+      </c>
+      <c r="C2" t="n">
+        <v>21</v>
+      </c>
+      <c r="D2" t="n">
+        <v>-0.09533377287767833</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-0.0944531088805954</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2020 Q2 → 2020 Q3</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.1530957378794786</v>
+      </c>
+      <c r="C3" t="n">
+        <v>22</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.009034153326759255</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.02279536523657228</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2020 Q3 → 2020 Q4</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.5250160645953914</v>
+      </c>
+      <c r="C4" t="n">
+        <v>24</v>
+      </c>
+      <c r="D4" t="n">
+        <v>-0.1149346188002442</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-0.114934618800244</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2020 Q4 → 2021 Q1</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.0001406334165718892</v>
+      </c>
+      <c r="C5" t="n">
+        <v>24</v>
+      </c>
+      <c r="D5" t="n">
+        <v>-0.1153731613716841</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.04259347349587472</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2021 Q1 → 2021 Q2</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.06052581235763232</v>
+      </c>
+      <c r="C6" t="n">
+        <v>37</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-0.02865720304700771</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-0.02450378798577472</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2021 Q2 → 2021 Q3</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.05454257640255189</v>
+      </c>
+      <c r="C7" t="n">
+        <v>40</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-0.04563704519217358</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-0.04350852781587513</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2021 Q3 → 2021 Q4</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.0390696750155638</v>
+      </c>
+      <c r="C8" t="n">
+        <v>43</v>
+      </c>
+      <c r="D8" t="n">
+        <v>-0.0823076788463572</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-0.05807081975649583</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2021 Q4 → 2022 Q1</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.1779162126349572</v>
+      </c>
+      <c r="C9" t="n">
+        <v>47</v>
+      </c>
+      <c r="D9" t="n">
+        <v>-0.1212985618345097</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-0.06013744244466211</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2022 Q1 → 2022 Q2</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.003177645600907497</v>
+      </c>
+      <c r="C10" t="n">
+        <v>61</v>
+      </c>
+      <c r="D10" t="n">
+        <v>-0.08249549922554951</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-0.07004683672180403</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2022 Q2 → 2022 Q3</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.02379507950733128</v>
+      </c>
+      <c r="C11" t="n">
+        <v>67</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-0.07047599670974297</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-0.05261869089809537</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2022 Q3 → 2022 Q4</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.1669482208429905</v>
+      </c>
+      <c r="C12" t="n">
+        <v>71</v>
+      </c>
+      <c r="D12" t="n">
+        <v>-0.1243246018710703</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-0.06262269532608714</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2022 Q4 → 2023 Q1</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.1645733661052395</v>
+      </c>
+      <c r="C13" t="n">
+        <v>85</v>
+      </c>
+      <c r="D13" t="n">
+        <v>-0.06910333115948455</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-0.05392463511235614</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2023 Q1 → 2023 Q2</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.0402926431341275</v>
+      </c>
+      <c r="C14" t="n">
+        <v>90</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-0.0389179069905778</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-0.01126856209562319</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2023 Q2 → 2023 Q3</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.01140763876668138</v>
+      </c>
+      <c r="C15" t="n">
+        <v>99</v>
+      </c>
+      <c r="D15" t="n">
+        <v>-0.0334622127153237</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-0.02389111380447295</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2023 Q3 → 2023 Q4</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.01522942958702034</v>
+      </c>
+      <c r="C16" t="n">
+        <v>102</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-0.1019201054308967</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-0.05922527162814977</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2023 Q4 → 2024 Q1</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.09701187393461386</v>
+      </c>
+      <c r="C17" t="n">
+        <v>116</v>
+      </c>
+      <c r="D17" t="n">
+        <v>-0.08979187724887154</v>
+      </c>
+      <c r="E17" t="n">
+        <v>-0.07256325532505148</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2024 Q1 → 2024 Q2</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.167664143010763</v>
+      </c>
+      <c r="C18" t="n">
+        <v>121</v>
+      </c>
+      <c r="D18" t="n">
+        <v>-0.05472115511075102</v>
+      </c>
+      <c r="E18" t="n">
+        <v>-0.05051527317568803</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2024 Q2 → 2024 Q3</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.1312478047022526</v>
+      </c>
+      <c r="C19" t="n">
+        <v>127</v>
+      </c>
+      <c r="D19" t="n">
+        <v>-0.0134879315657925</v>
+      </c>
+      <c r="E19" t="n">
+        <v>-0.009883492260612718</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2024 Q3 → 2024 Q4</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0.000431006805845402</v>
+      </c>
+      <c r="C20" t="n">
+        <v>128</v>
+      </c>
+      <c r="D20" t="n">
+        <v>-0.0320894454578143</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.004954756198602965</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2024 Q4 → 2025 Q1</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.0911331186494142</v>
+      </c>
+      <c r="C21" t="n">
+        <v>138</v>
+      </c>
+      <c r="D21" t="n">
+        <v>-0.08255872174578359</v>
+      </c>
+      <c r="E21" t="n">
+        <v>-0.07723614723735492</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2025 Q1 → 2025 Q2</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0.03822939752849597</v>
+      </c>
+      <c r="C22" t="n">
+        <v>131</v>
+      </c>
+      <c r="D22" t="n">
+        <v>-0.0352582333112843</v>
+      </c>
+      <c r="E22" t="n">
+        <v>-0.03183427134739731</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Overall (Average)</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>0.1278790618288475</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1594</v>
+      </c>
+      <c r="D23" t="n">
+        <v>-0.06776737653265896</v>
+      </c>
+      <c r="E23" t="n">
+        <v>-0.04289975979453764</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>